<commit_message>
Record 2026-09-02 NAR and kyotei predictions in local Excel.
Fill the 202609 sheets after merging PR #6. JRA had no meeting.
Drive sync was not possible without credentials.

Co-authored-by: tama357 <tama357@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/個人予想/excel/地方競馬_予想記入シート_2026年9月.xlsx
+++ b/個人予想/excel/地方競馬_予想記入シート_2026年9月.xlsx
@@ -1237,15 +1237,47 @@
       <c r="B8" s="40" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="41" t="n"/>
-      <c r="D8" s="41" t="n"/>
-      <c r="E8" s="41" t="n"/>
-      <c r="F8" s="77" t="n"/>
-      <c r="G8" s="78" t="n"/>
-      <c r="H8" s="42" t="n"/>
-      <c r="I8" s="42" t="n"/>
-      <c r="J8" s="79" t="n"/>
-      <c r="K8" s="42" t="n"/>
+      <c r="C8" s="41" t="inlineStr">
+        <is>
+          <t>中穴</t>
+        </is>
+      </c>
+      <c r="D8" s="41" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E8" s="41" t="inlineStr">
+        <is>
+          <t>園田</t>
+        </is>
+      </c>
+      <c r="F8" s="77" t="n">
+        <v>10</v>
+      </c>
+      <c r="G8" s="78" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="H8" s="42" t="inlineStr">
+        <is>
+          <t>4-2-35678</t>
+        </is>
+      </c>
+      <c r="I8" s="42" t="inlineStr">
+        <is>
+          <t>4-1-35678 4-3-5678</t>
+        </is>
+      </c>
+      <c r="J8" s="79" t="n">
+        <v>14</v>
+      </c>
+      <c r="K8" s="42" t="inlineStr">
+        <is>
+          <t>[予想しやすさ83] 軸4番。nar.netkeiba race_id=202650090210 軸4番ゼットカレン（4番人気） / 想定:ゼットカレン（4番）中心。相手2・1 / リスク:展開変化に注意</t>
+        </is>
+      </c>
       <c r="L8" s="43" t="n"/>
       <c r="M8" s="80" t="n"/>
       <c r="N8" s="44" t="inlineStr">
@@ -1259,15 +1291,47 @@
       <c r="B9" s="33" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="35" t="n"/>
-      <c r="D9" s="35" t="n"/>
-      <c r="E9" s="35" t="n"/>
-      <c r="F9" s="82" t="n"/>
-      <c r="G9" s="83" t="n"/>
-      <c r="H9" s="36" t="n"/>
-      <c r="I9" s="36" t="n"/>
-      <c r="J9" s="84" t="n"/>
-      <c r="K9" s="36" t="n"/>
+      <c r="C9" s="35" t="inlineStr">
+        <is>
+          <t>中穴</t>
+        </is>
+      </c>
+      <c r="D9" s="35" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E9" s="35" t="inlineStr">
+        <is>
+          <t>名古屋</t>
+        </is>
+      </c>
+      <c r="F9" s="82" t="n">
+        <v>9</v>
+      </c>
+      <c r="G9" s="83" t="inlineStr">
+        <is>
+          <t>18:55</t>
+        </is>
+      </c>
+      <c r="H9" s="36" t="inlineStr">
+        <is>
+          <t>2-3-14678</t>
+        </is>
+      </c>
+      <c r="I9" s="36" t="inlineStr">
+        <is>
+          <t>2-9-14678 2-1-4678</t>
+        </is>
+      </c>
+      <c r="J9" s="84" t="n">
+        <v>14</v>
+      </c>
+      <c r="K9" s="36" t="inlineStr">
+        <is>
+          <t>[予想しやすさ80] 軸2番。nar.netkeiba race_id=202648090209 軸2番ヒオウギ（4番人気） / 想定:ヒオウギ（2番）中心。相手3・9 / リスク:展開変化に注意</t>
+        </is>
+      </c>
       <c r="L9" s="38" t="n"/>
       <c r="M9" s="85" t="n"/>
       <c r="N9" s="46" t="inlineStr">
@@ -1281,15 +1345,47 @@
       <c r="B10" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="C10" s="35" t="n"/>
-      <c r="D10" s="35" t="n"/>
-      <c r="E10" s="35" t="n"/>
-      <c r="F10" s="82" t="n"/>
-      <c r="G10" s="83" t="n"/>
-      <c r="H10" s="36" t="n"/>
-      <c r="I10" s="36" t="n"/>
-      <c r="J10" s="84" t="n"/>
-      <c r="K10" s="36" t="n"/>
+      <c r="C10" s="35" t="inlineStr">
+        <is>
+          <t>中穴</t>
+        </is>
+      </c>
+      <c r="D10" s="35" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E10" s="35" t="inlineStr">
+        <is>
+          <t>名古屋</t>
+        </is>
+      </c>
+      <c r="F10" s="82" t="n">
+        <v>10</v>
+      </c>
+      <c r="G10" s="83" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="H10" s="36" t="inlineStr">
+        <is>
+          <t>7-3-124689</t>
+        </is>
+      </c>
+      <c r="I10" s="36" t="inlineStr">
+        <is>
+          <t>7-5-124689</t>
+        </is>
+      </c>
+      <c r="J10" s="84" t="n">
+        <v>12</v>
+      </c>
+      <c r="K10" s="36" t="inlineStr">
+        <is>
+          <t>[予想しやすさ80] 軸7番。nar.netkeiba race_id=202648090210 軸7番ワールドキッス（4番人気） / 想定:ワールドキッス（7番）中心。相手3・5 / リスク:wide_open</t>
+        </is>
+      </c>
       <c r="L10" s="38" t="n"/>
       <c r="M10" s="85" t="n"/>
       <c r="N10" s="46" t="inlineStr">
@@ -1303,15 +1399,47 @@
       <c r="B11" s="33" t="n">
         <v>4</v>
       </c>
-      <c r="C11" s="35" t="n"/>
-      <c r="D11" s="35" t="n"/>
-      <c r="E11" s="35" t="n"/>
-      <c r="F11" s="82" t="n"/>
-      <c r="G11" s="83" t="n"/>
-      <c r="H11" s="36" t="n"/>
-      <c r="I11" s="36" t="n"/>
-      <c r="J11" s="84" t="n"/>
-      <c r="K11" s="36" t="n"/>
+      <c r="C11" s="35" t="inlineStr">
+        <is>
+          <t>中穴</t>
+        </is>
+      </c>
+      <c r="D11" s="35" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E11" s="35" t="inlineStr">
+        <is>
+          <t>名古屋</t>
+        </is>
+      </c>
+      <c r="F11" s="82" t="n">
+        <v>11</v>
+      </c>
+      <c r="G11" s="83" t="inlineStr">
+        <is>
+          <t>20:05</t>
+        </is>
+      </c>
+      <c r="H11" s="36" t="inlineStr">
+        <is>
+          <t>4-6-123589</t>
+        </is>
+      </c>
+      <c r="I11" s="36" t="inlineStr">
+        <is>
+          <t>4-7-123589</t>
+        </is>
+      </c>
+      <c r="J11" s="84" t="n">
+        <v>12</v>
+      </c>
+      <c r="K11" s="36" t="inlineStr">
+        <is>
+          <t>[予想しやすさ80] 軸4番。nar.netkeiba race_id=202648090211 軸4番バルサミコ（4番人気） / 想定:バルサミコ（4番）中心。相手6・7 / リスク:wide_open</t>
+        </is>
+      </c>
       <c r="L11" s="38" t="n"/>
       <c r="M11" s="85" t="n"/>
       <c r="N11" s="46" t="inlineStr">
@@ -1325,15 +1453,47 @@
       <c r="B12" s="48" t="n">
         <v>5</v>
       </c>
-      <c r="C12" s="49" t="n"/>
-      <c r="D12" s="49" t="n"/>
-      <c r="E12" s="49" t="n"/>
-      <c r="F12" s="87" t="n"/>
-      <c r="G12" s="88" t="n"/>
-      <c r="H12" s="50" t="n"/>
-      <c r="I12" s="50" t="n"/>
-      <c r="J12" s="89" t="n"/>
-      <c r="K12" s="50" t="n"/>
+      <c r="C12" s="49" t="inlineStr">
+        <is>
+          <t>中穴</t>
+        </is>
+      </c>
+      <c r="D12" s="49" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E12" s="49" t="inlineStr">
+        <is>
+          <t>名古屋</t>
+        </is>
+      </c>
+      <c r="F12" s="87" t="n">
+        <v>12</v>
+      </c>
+      <c r="G12" s="88" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="H12" s="50" t="inlineStr">
+        <is>
+          <t>6-8-124579</t>
+        </is>
+      </c>
+      <c r="I12" s="50" t="inlineStr">
+        <is>
+          <t>6-3-124579</t>
+        </is>
+      </c>
+      <c r="J12" s="89" t="n">
+        <v>12</v>
+      </c>
+      <c r="K12" s="50" t="inlineStr">
+        <is>
+          <t>[予想しやすさ80] 軸6番。nar.netkeiba race_id=202648090212 軸6番メイショウバルキア（4番人気） / 想定:メイショウバルキア（6番）中心。相手8・3 / リスク:wide_open</t>
+        </is>
+      </c>
       <c r="L12" s="51" t="n"/>
       <c r="M12" s="90" t="n"/>
       <c r="N12" s="52" t="inlineStr">

</xml_diff>